<commit_message>
fix(sb): integer rounding on operator-Excel SB ingestion path too
sb_ingest_from_api.py already rounds Impressions/Clicks/Units to int
after distribution (added in the sales-weighted commit).  sb_ingest.py
(the operator-exported Excel path used for W21) was still emitting
fractional values like 79157.55 -- which display rounds in the UI but
leaks fractional into CSV / XLSX exports.

Same rounding rule now applied uniformly: event-count columns
(Impressions, Clicks, 14 Day Total Units) round to int after the final
per-(Portfolio, Campaign, ASIN, Brand) groupby.  Spend and Sales stay
float since rupee amounts legitimately carry paise.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
@@ -18668,7 +18668,7 @@
         <v>5568.860000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>2.333333333333333</v>
+        <v>2</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -18705,7 +18705,7 @@
         <v>5568.860000000001</v>
       </c>
       <c r="H5" t="n">
-        <v>2.333333333333333</v>
+        <v>2</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -18742,7 +18742,7 @@
         <v>5568.860000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>2.333333333333333</v>
+        <v>2</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -18807,7 +18807,7 @@
         <v>9326</v>
       </c>
       <c r="E8" t="n">
-        <v>79.33333333333333</v>
+        <v>79</v>
       </c>
       <c r="F8" t="n">
         <v>1333.07</v>
@@ -18816,7 +18816,7 @@
         <v>6368.923333333335</v>
       </c>
       <c r="H8" t="n">
-        <v>4.666666666666667</v>
+        <v>5</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -18844,7 +18844,7 @@
         <v>9326</v>
       </c>
       <c r="E9" t="n">
-        <v>79.33333333333333</v>
+        <v>79</v>
       </c>
       <c r="F9" t="n">
         <v>1333.07</v>
@@ -18853,7 +18853,7 @@
         <v>6368.923333333335</v>
       </c>
       <c r="H9" t="n">
-        <v>4.666666666666667</v>
+        <v>5</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -18881,7 +18881,7 @@
         <v>9326</v>
       </c>
       <c r="E10" t="n">
-        <v>79.33333333333333</v>
+        <v>79</v>
       </c>
       <c r="F10" t="n">
         <v>1333.07</v>
@@ -18890,7 +18890,7 @@
         <v>6368.923333333335</v>
       </c>
       <c r="H10" t="n">
-        <v>4.666666666666667</v>
+        <v>5</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -18915,10 +18915,10 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E11" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F11" t="n">
         <v>542.6024137931034</v>
@@ -18927,7 +18927,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H11" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -18952,10 +18952,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E12" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F12" t="n">
         <v>542.6024137931034</v>
@@ -18964,7 +18964,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -18989,10 +18989,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E13" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F13" t="n">
         <v>542.6024137931034</v>
@@ -19001,7 +19001,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H13" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -19026,10 +19026,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E14" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F14" t="n">
         <v>542.6024137931034</v>
@@ -19038,7 +19038,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H14" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -19063,10 +19063,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E15" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F15" t="n">
         <v>542.6024137931034</v>
@@ -19075,7 +19075,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H15" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -19100,10 +19100,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E16" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F16" t="n">
         <v>542.6024137931034</v>
@@ -19112,7 +19112,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H16" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -19137,10 +19137,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E17" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F17" t="n">
         <v>542.6024137931034</v>
@@ -19149,7 +19149,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H17" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -19174,10 +19174,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E18" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F18" t="n">
         <v>542.6024137931034</v>
@@ -19186,7 +19186,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H18" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -19211,10 +19211,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E19" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F19" t="n">
         <v>542.6024137931034</v>
@@ -19223,7 +19223,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H19" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -19248,10 +19248,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E20" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F20" t="n">
         <v>542.6024137931034</v>
@@ -19260,7 +19260,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H20" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -19285,10 +19285,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E21" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F21" t="n">
         <v>542.6024137931034</v>
@@ -19297,7 +19297,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H21" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -19322,10 +19322,10 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E22" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F22" t="n">
         <v>542.6024137931034</v>
@@ -19334,7 +19334,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H22" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -19359,10 +19359,10 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E23" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F23" t="n">
         <v>542.6024137931034</v>
@@ -19371,7 +19371,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H23" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -19396,10 +19396,10 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E24" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F24" t="n">
         <v>542.6024137931034</v>
@@ -19408,7 +19408,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H24" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -19433,10 +19433,10 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E25" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F25" t="n">
         <v>542.6024137931034</v>
@@ -19445,7 +19445,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H25" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -19470,10 +19470,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E26" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F26" t="n">
         <v>542.6024137931034</v>
@@ -19482,7 +19482,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H26" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -19507,10 +19507,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E27" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F27" t="n">
         <v>542.6024137931034</v>
@@ -19519,7 +19519,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H27" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -19544,10 +19544,10 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E28" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F28" t="n">
         <v>542.6024137931034</v>
@@ -19556,7 +19556,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H28" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -19581,10 +19581,10 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E29" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F29" t="n">
         <v>542.6024137931034</v>
@@ -19593,7 +19593,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H29" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -19618,10 +19618,10 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E30" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F30" t="n">
         <v>542.6024137931034</v>
@@ -19630,7 +19630,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H30" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -19655,10 +19655,10 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E31" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F31" t="n">
         <v>542.6024137931034</v>
@@ -19667,7 +19667,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H31" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -19692,10 +19692,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E32" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F32" t="n">
         <v>542.6024137931034</v>
@@ -19704,7 +19704,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H32" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -19729,10 +19729,10 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E33" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F33" t="n">
         <v>542.6024137931034</v>
@@ -19741,7 +19741,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H33" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -19766,10 +19766,10 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E34" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F34" t="n">
         <v>542.6024137931034</v>
@@ -19778,7 +19778,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H34" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -19803,10 +19803,10 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E35" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F35" t="n">
         <v>542.6024137931034</v>
@@ -19815,7 +19815,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H35" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -19840,10 +19840,10 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E36" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F36" t="n">
         <v>542.6024137931034</v>
@@ -19852,7 +19852,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H36" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -19877,10 +19877,10 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E37" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F37" t="n">
         <v>542.6024137931034</v>
@@ -19889,7 +19889,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H37" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -19914,10 +19914,10 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E38" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F38" t="n">
         <v>542.6024137931034</v>
@@ -19926,7 +19926,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H38" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -19951,10 +19951,10 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>7178.551724137931</v>
+        <v>7179</v>
       </c>
       <c r="E39" t="n">
-        <v>29.68965517241379</v>
+        <v>30</v>
       </c>
       <c r="F39" t="n">
         <v>542.6024137931034</v>
@@ -19963,7 +19963,7 @@
         <v>1054.763448275862</v>
       </c>
       <c r="H39" t="n">
-        <v>0.5172413793103449</v>
+        <v>1</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-05-31
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1142.02</v>
+        <v>1132.9</v>
       </c>
       <c r="E5" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F5" t="n">
-        <v>17329</v>
+        <v>17323</v>
       </c>
       <c r="G5" t="n">
         <v>3261.86</v>
@@ -759,7 +759,7 @@
         <v>32</v>
       </c>
       <c r="F12" t="n">
-        <v>4378</v>
+        <v>4377</v>
       </c>
       <c r="G12" t="n">
         <v>3388.13</v>
@@ -815,7 +815,7 @@
         <v>56</v>
       </c>
       <c r="F14" t="n">
-        <v>7165</v>
+        <v>7164</v>
       </c>
       <c r="G14" t="n">
         <v>1355.08</v>
@@ -927,7 +927,7 @@
         <v>16</v>
       </c>
       <c r="F18" t="n">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -1291,7 +1291,7 @@
         <v>36</v>
       </c>
       <c r="F31" t="n">
-        <v>13155</v>
+        <v>13154</v>
       </c>
       <c r="G31" t="n">
         <v>2287.29</v>
@@ -1459,7 +1459,7 @@
         <v>157</v>
       </c>
       <c r="F37" t="n">
-        <v>32893</v>
+        <v>32881</v>
       </c>
       <c r="G37" t="n">
         <v>5167.8</v>
@@ -1487,7 +1487,7 @@
         <v>226</v>
       </c>
       <c r="F38" t="n">
-        <v>36356</v>
+        <v>36344</v>
       </c>
       <c r="G38" t="n">
         <v>1312.71</v>
@@ -1515,7 +1515,7 @@
         <v>145</v>
       </c>
       <c r="F39" t="n">
-        <v>29638</v>
+        <v>29632</v>
       </c>
       <c r="G39" t="n">
         <v>1312.71</v>
@@ -1537,13 +1537,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1744.36</v>
+        <v>1741.32</v>
       </c>
       <c r="E40" t="n">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F40" t="n">
-        <v>22539</v>
+        <v>22516</v>
       </c>
       <c r="G40" t="n">
         <v>12709.32</v>
@@ -1683,7 +1683,7 @@
         <v>246</v>
       </c>
       <c r="F45" t="n">
-        <v>41015</v>
+        <v>41010</v>
       </c>
       <c r="G45" t="n">
         <v>5082.209999999999</v>
@@ -1851,7 +1851,7 @@
         <v>65</v>
       </c>
       <c r="F51" t="n">
-        <v>15525</v>
+        <v>15524</v>
       </c>
       <c r="G51" t="n">
         <v>6734.76</v>
@@ -1935,7 +1935,7 @@
         <v>139</v>
       </c>
       <c r="F54" t="n">
-        <v>15113</v>
+        <v>15112</v>
       </c>
       <c r="G54" t="n">
         <v>4489.84</v>
@@ -1957,13 +1957,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>3019.62</v>
+        <v>2988.83</v>
       </c>
       <c r="E55" t="n">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="F55" t="n">
-        <v>26367</v>
+        <v>26358</v>
       </c>
       <c r="G55" t="n">
         <v>21178.85</v>
@@ -2019,7 +2019,7 @@
         <v>925</v>
       </c>
       <c r="F57" t="n">
-        <v>78887</v>
+        <v>78884</v>
       </c>
       <c r="G57" t="n">
         <v>53679.75</v>
@@ -2125,13 +2125,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1780.04</v>
+        <v>1773.58</v>
       </c>
       <c r="E61" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F61" t="n">
-        <v>22915</v>
+        <v>22910</v>
       </c>
       <c r="G61" t="n">
         <v>6438.99</v>
@@ -2159,7 +2159,7 @@
         <v>53</v>
       </c>
       <c r="F62" t="n">
-        <v>7115</v>
+        <v>7110</v>
       </c>
       <c r="G62" t="n">
         <v>6395.76</v>
@@ -2299,7 +2299,7 @@
         <v>85</v>
       </c>
       <c r="F67" t="n">
-        <v>17329</v>
+        <v>17328</v>
       </c>
       <c r="G67" t="n">
         <v>823.73</v>
@@ -2439,7 +2439,7 @@
         <v>112</v>
       </c>
       <c r="F72" t="n">
-        <v>13670</v>
+        <v>13668</v>
       </c>
       <c r="G72" t="n">
         <v>9843.200000000001</v>
@@ -2523,7 +2523,7 @@
         <v>265</v>
       </c>
       <c r="F75" t="n">
-        <v>70966</v>
+        <v>70954</v>
       </c>
       <c r="G75" t="n">
         <v>0</v>
@@ -2635,7 +2635,7 @@
         <v>326</v>
       </c>
       <c r="F79" t="n">
-        <v>39859</v>
+        <v>39846</v>
       </c>
       <c r="G79" t="n">
         <v>39652.55</v>
@@ -2685,13 +2685,13 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>5278.01</v>
+        <v>5265.04</v>
       </c>
       <c r="E81" t="n">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="F81" t="n">
-        <v>73911</v>
+        <v>73905</v>
       </c>
       <c r="G81" t="n">
         <v>43513.23</v>
@@ -2719,7 +2719,7 @@
         <v>242</v>
       </c>
       <c r="F82" t="n">
-        <v>21945</v>
+        <v>21941</v>
       </c>
       <c r="G82" t="n">
         <v>24401.7</v>
@@ -2769,13 +2769,13 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>12694.97</v>
+        <v>12686.34</v>
       </c>
       <c r="E84" t="n">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="F84" t="n">
-        <v>96382</v>
+        <v>96377</v>
       </c>
       <c r="G84" t="n">
         <v>52900.00999999999</v>
@@ -2943,7 +2943,7 @@
         <v>126</v>
       </c>
       <c r="F90" t="n">
-        <v>8148</v>
+        <v>8147</v>
       </c>
       <c r="G90" t="n">
         <v>2456.78</v>
@@ -3027,7 +3027,7 @@
         <v>179</v>
       </c>
       <c r="F93" t="n">
-        <v>30065</v>
+        <v>30058</v>
       </c>
       <c r="G93" t="n">
         <v>6353.400000000001</v>
@@ -3049,13 +3049,13 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>2683.18</v>
+        <v>2677.41</v>
       </c>
       <c r="E94" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F94" t="n">
-        <v>27047</v>
+        <v>27042</v>
       </c>
       <c r="G94" t="n">
         <v>15816.96</v>
@@ -3083,7 +3083,7 @@
         <v>36</v>
       </c>
       <c r="F95" t="n">
-        <v>2270</v>
+        <v>2269</v>
       </c>
       <c r="G95" t="n">
         <v>2117.8</v>
@@ -3139,7 +3139,7 @@
         <v>85</v>
       </c>
       <c r="F97" t="n">
-        <v>10839</v>
+        <v>10837</v>
       </c>
       <c r="G97" t="n">
         <v>12953.43</v>
@@ -3329,13 +3329,13 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>3062.05</v>
+        <v>3056.28</v>
       </c>
       <c r="E104" t="n">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="F104" t="n">
-        <v>134758</v>
+        <v>134753</v>
       </c>
       <c r="G104" t="n">
         <v>2626.27</v>
@@ -3419,7 +3419,7 @@
         <v>174</v>
       </c>
       <c r="F107" t="n">
-        <v>14357</v>
+        <v>14356</v>
       </c>
       <c r="G107" t="n">
         <v>4726.259999999999</v>
@@ -3475,7 +3475,7 @@
         <v>17</v>
       </c>
       <c r="F109" t="n">
-        <v>3900</v>
+        <v>3899</v>
       </c>
       <c r="G109" t="n">
         <v>2015.25</v>
@@ -3531,7 +3531,7 @@
         <v>34</v>
       </c>
       <c r="F111" t="n">
-        <v>6035</v>
+        <v>6033</v>
       </c>
       <c r="G111" t="n">
         <v>0</v>
@@ -3615,7 +3615,7 @@
         <v>66</v>
       </c>
       <c r="F114" t="n">
-        <v>23565</v>
+        <v>23562</v>
       </c>
       <c r="G114" t="n">
         <v>5761.02</v>
@@ -3643,7 +3643,7 @@
         <v>26</v>
       </c>
       <c r="F115" t="n">
-        <v>2907</v>
+        <v>2906</v>
       </c>
       <c r="G115" t="n">
         <v>4405.93</v>
@@ -3665,13 +3665,13 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>860.02</v>
+        <v>853.78</v>
       </c>
       <c r="E116" t="n">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F116" t="n">
-        <v>10038</v>
+        <v>10033</v>
       </c>
       <c r="G116" t="n">
         <v>1488.98</v>
@@ -3693,13 +3693,13 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>2996.97</v>
+        <v>2992.93</v>
       </c>
       <c r="E117" t="n">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F117" t="n">
-        <v>12313</v>
+        <v>12312</v>
       </c>
       <c r="G117" t="n">
         <v>10845.76</v>
@@ -3749,13 +3749,13 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>7820.08</v>
+        <v>7818.139999999999</v>
       </c>
       <c r="E119" t="n">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="F119" t="n">
-        <v>72900</v>
+        <v>72888</v>
       </c>
       <c r="G119" t="n">
         <v>54107.63</v>
@@ -3783,7 +3783,7 @@
         <v>585</v>
       </c>
       <c r="F120" t="n">
-        <v>81215</v>
+        <v>81210</v>
       </c>
       <c r="G120" t="n">
         <v>12355.92</v>
@@ -3867,7 +3867,7 @@
         <v>358</v>
       </c>
       <c r="F123" t="n">
-        <v>76050</v>
+        <v>76047</v>
       </c>
       <c r="G123" t="n">
         <v>8487.289999999999</v>
@@ -3923,7 +3923,7 @@
         <v>112</v>
       </c>
       <c r="F125" t="n">
-        <v>26296</v>
+        <v>26290</v>
       </c>
       <c r="G125" t="n">
         <v>6689.82</v>
@@ -3951,7 +3951,7 @@
         <v>63</v>
       </c>
       <c r="F126" t="n">
-        <v>12866</v>
+        <v>12861</v>
       </c>
       <c r="G126" t="n">
         <v>5088.98</v>
@@ -3979,7 +3979,7 @@
         <v>20</v>
       </c>
       <c r="F127" t="n">
-        <v>4626</v>
+        <v>4621</v>
       </c>
       <c r="G127" t="n">
         <v>0</v>
@@ -4063,7 +4063,7 @@
         <v>39</v>
       </c>
       <c r="F130" t="n">
-        <v>2867</v>
+        <v>2866</v>
       </c>
       <c r="G130" t="n">
         <v>0</v>
@@ -4113,13 +4113,13 @@
         </is>
       </c>
       <c r="D132" t="n">
-        <v>4180.17</v>
+        <v>4177.29</v>
       </c>
       <c r="E132" t="n">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="F132" t="n">
-        <v>59352</v>
+        <v>59338</v>
       </c>
       <c r="G132" t="n">
         <v>12556.78</v>
@@ -4141,13 +4141,13 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>4979.78</v>
+        <v>4977.16</v>
       </c>
       <c r="E133" t="n">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="F133" t="n">
-        <v>8986</v>
+        <v>8983</v>
       </c>
       <c r="G133" t="n">
         <v>27295.72</v>
@@ -4231,7 +4231,7 @@
         <v>125</v>
       </c>
       <c r="F136" t="n">
-        <v>17461</v>
+        <v>17458</v>
       </c>
       <c r="G136" t="n">
         <v>0</v>
@@ -4253,13 +4253,13 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>9498.02</v>
+        <v>9489.98</v>
       </c>
       <c r="E137" t="n">
-        <v>839</v>
+        <v>837</v>
       </c>
       <c r="F137" t="n">
-        <v>82989</v>
+        <v>82975</v>
       </c>
       <c r="G137" t="n">
         <v>54907.65</v>
@@ -4287,7 +4287,7 @@
         <v>606</v>
       </c>
       <c r="F138" t="n">
-        <v>45311</v>
+        <v>45307</v>
       </c>
       <c r="G138" t="n">
         <v>34739</v>
@@ -4309,13 +4309,13 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>3294.18</v>
+        <v>3290.72</v>
       </c>
       <c r="E139" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F139" t="n">
-        <v>12322</v>
+        <v>12320</v>
       </c>
       <c r="G139" t="n">
         <v>0</v>
@@ -4455,7 +4455,7 @@
         <v>334</v>
       </c>
       <c r="F144" t="n">
-        <v>49062</v>
+        <v>49059</v>
       </c>
       <c r="G144" t="n">
         <v>0</v>
@@ -4483,7 +4483,7 @@
         <v>184</v>
       </c>
       <c r="F145" t="n">
-        <v>37515</v>
+        <v>37510</v>
       </c>
       <c r="G145" t="n">
         <v>3388.98</v>
@@ -4511,7 +4511,7 @@
         <v>18</v>
       </c>
       <c r="F146" t="n">
-        <v>9144</v>
+        <v>9141</v>
       </c>
       <c r="G146" t="n">
         <v>0</v>
@@ -4533,13 +4533,13 @@
         </is>
       </c>
       <c r="D147" t="n">
-        <v>461.91</v>
+        <v>450.13</v>
       </c>
       <c r="E147" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F147" t="n">
-        <v>5321</v>
+        <v>5317</v>
       </c>
       <c r="G147" t="n">
         <v>2244.92</v>
@@ -4567,7 +4567,7 @@
         <v>87</v>
       </c>
       <c r="F148" t="n">
-        <v>12822</v>
+        <v>12821</v>
       </c>
       <c r="G148" t="n">
         <v>3938.98</v>
@@ -4595,7 +4595,7 @@
         <v>63</v>
       </c>
       <c r="F149" t="n">
-        <v>11746</v>
+        <v>11744</v>
       </c>
       <c r="G149" t="n">
         <v>2625.42</v>
@@ -4623,7 +4623,7 @@
         <v>57</v>
       </c>
       <c r="F150" t="n">
-        <v>12465</v>
+        <v>12463</v>
       </c>
       <c r="G150" t="n">
         <v>4574.57</v>
@@ -4645,13 +4645,13 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>2292.43</v>
+        <v>2288.38</v>
       </c>
       <c r="E151" t="n">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F151" t="n">
-        <v>20683</v>
+        <v>20678</v>
       </c>
       <c r="G151" t="n">
         <v>7879.660000000001</v>
@@ -4707,7 +4707,7 @@
         <v>106</v>
       </c>
       <c r="F153" t="n">
-        <v>6655</v>
+        <v>6653</v>
       </c>
       <c r="G153" t="n">
         <v>0</v>
@@ -4847,7 +4847,7 @@
         <v>53</v>
       </c>
       <c r="F158" t="n">
-        <v>9952</v>
+        <v>9951</v>
       </c>
       <c r="G158" t="n">
         <v>6523.72</v>
@@ -4959,7 +4959,7 @@
         <v>169</v>
       </c>
       <c r="F162" t="n">
-        <v>34222</v>
+        <v>34221</v>
       </c>
       <c r="G162" t="n">
         <v>4490.68</v>
@@ -5211,7 +5211,7 @@
         <v>4</v>
       </c>
       <c r="F171" t="n">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="G171" t="n">
         <v>0</v>
@@ -5239,7 +5239,7 @@
         <v>15</v>
       </c>
       <c r="F172" t="n">
-        <v>2882</v>
+        <v>2880</v>
       </c>
       <c r="G172" t="n">
         <v>0</v>
@@ -5603,7 +5603,7 @@
         <v>33</v>
       </c>
       <c r="F185" t="n">
-        <v>2847</v>
+        <v>2846</v>
       </c>
       <c r="G185" t="n">
         <v>3727.12</v>
@@ -5631,7 +5631,7 @@
         <v>50</v>
       </c>
       <c r="F186" t="n">
-        <v>2985</v>
+        <v>2982</v>
       </c>
       <c r="G186" t="n">
         <v>0</v>
@@ -5659,7 +5659,7 @@
         <v>0</v>
       </c>
       <c r="F187" t="n">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="G187" t="n">
         <v>0</v>
@@ -5687,7 +5687,7 @@
         <v>1</v>
       </c>
       <c r="F188" t="n">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="G188" t="n">
         <v>0</v>
@@ -5771,7 +5771,7 @@
         <v>304</v>
       </c>
       <c r="F191" t="n">
-        <v>59529</v>
+        <v>59527</v>
       </c>
       <c r="G191" t="n">
         <v>0</v>
@@ -5855,7 +5855,7 @@
         <v>97</v>
       </c>
       <c r="F194" t="n">
-        <v>60036</v>
+        <v>60030</v>
       </c>
       <c r="G194" t="n">
         <v>6734.76</v>
@@ -5883,7 +5883,7 @@
         <v>29</v>
       </c>
       <c r="F195" t="n">
-        <v>10709</v>
+        <v>10707</v>
       </c>
       <c r="G195" t="n">
         <v>2244.92</v>
@@ -5911,7 +5911,7 @@
         <v>15</v>
       </c>
       <c r="F196" t="n">
-        <v>8731</v>
+        <v>8719</v>
       </c>
       <c r="G196" t="n">
         <v>4066.95</v>
@@ -5939,7 +5939,7 @@
         <v>9</v>
       </c>
       <c r="F197" t="n">
-        <v>2356</v>
+        <v>2351</v>
       </c>
       <c r="G197" t="n">
         <v>0</v>
@@ -5967,7 +5967,7 @@
         <v>28</v>
       </c>
       <c r="F198" t="n">
-        <v>2718</v>
+        <v>2716</v>
       </c>
       <c r="G198" t="n">
         <v>0</v>
@@ -5995,7 +5995,7 @@
         <v>27</v>
       </c>
       <c r="F199" t="n">
-        <v>3371</v>
+        <v>3363</v>
       </c>
       <c r="G199" t="n">
         <v>1863.56</v>
@@ -6023,7 +6023,7 @@
         <v>211</v>
       </c>
       <c r="F200" t="n">
-        <v>28955</v>
+        <v>28942</v>
       </c>
       <c r="G200" t="n">
         <v>465.25</v>
@@ -6051,7 +6051,7 @@
         <v>22</v>
       </c>
       <c r="F201" t="n">
-        <v>4072</v>
+        <v>4067</v>
       </c>
       <c r="G201" t="n">
         <v>3388.98</v>
@@ -6163,7 +6163,7 @@
         <v>43</v>
       </c>
       <c r="F205" t="n">
-        <v>14031</v>
+        <v>14025</v>
       </c>
       <c r="G205" t="n">
         <v>3818.64</v>
@@ -6191,7 +6191,7 @@
         <v>5</v>
       </c>
       <c r="F206" t="n">
-        <v>6726</v>
+        <v>6725</v>
       </c>
       <c r="G206" t="n">
         <v>0</v>
@@ -6213,13 +6213,13 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>387.65</v>
+        <v>386.65</v>
       </c>
       <c r="E207" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F207" t="n">
-        <v>8767</v>
+        <v>8764</v>
       </c>
       <c r="G207" t="n">
         <v>7497.46</v>
@@ -6247,7 +6247,7 @@
         <v>38</v>
       </c>
       <c r="F208" t="n">
-        <v>37583</v>
+        <v>37582</v>
       </c>
       <c r="G208" t="n">
         <v>0</v>
@@ -6303,7 +6303,7 @@
         <v>10</v>
       </c>
       <c r="F210" t="n">
-        <v>15398</v>
+        <v>15397</v>
       </c>
       <c r="G210" t="n">
         <v>550</v>
@@ -6331,7 +6331,7 @@
         <v>23</v>
       </c>
       <c r="F211" t="n">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="G211" t="n">
         <v>0</v>
@@ -6387,7 +6387,7 @@
         <v>48</v>
       </c>
       <c r="F213" t="n">
-        <v>12773</v>
+        <v>12772</v>
       </c>
       <c r="G213" t="n">
         <v>1355.08</v>
@@ -6415,7 +6415,7 @@
         <v>778</v>
       </c>
       <c r="F214" t="n">
-        <v>120004</v>
+        <v>119978</v>
       </c>
       <c r="G214" t="n">
         <v>17991.53</v>
@@ -6471,7 +6471,7 @@
         <v>12</v>
       </c>
       <c r="F216" t="n">
-        <v>2812</v>
+        <v>2810</v>
       </c>
       <c r="G216" t="n">
         <v>0</v>
@@ -6499,7 +6499,7 @@
         <v>9</v>
       </c>
       <c r="F217" t="n">
-        <v>1951</v>
+        <v>1946</v>
       </c>
       <c r="G217" t="n">
         <v>0</v>
@@ -6527,7 +6527,7 @@
         <v>18</v>
       </c>
       <c r="F218" t="n">
-        <v>2729</v>
+        <v>2721</v>
       </c>
       <c r="G218" t="n">
         <v>1384.75</v>
@@ -6583,7 +6583,7 @@
         <v>27</v>
       </c>
       <c r="F220" t="n">
-        <v>24876</v>
+        <v>24875</v>
       </c>
       <c r="G220" t="n">
         <v>3727.11</v>
@@ -6611,7 +6611,7 @@
         <v>18</v>
       </c>
       <c r="F221" t="n">
-        <v>1550</v>
+        <v>1549</v>
       </c>
       <c r="G221" t="n">
         <v>0</v>
@@ -6639,7 +6639,7 @@
         <v>12</v>
       </c>
       <c r="F222" t="n">
-        <v>3163</v>
+        <v>3162</v>
       </c>
       <c r="G222" t="n">
         <v>0</v>
@@ -6667,7 +6667,7 @@
         <v>87</v>
       </c>
       <c r="F223" t="n">
-        <v>17578</v>
+        <v>17573</v>
       </c>
       <c r="G223" t="n">
         <v>9573.73</v>
@@ -6695,7 +6695,7 @@
         <v>24</v>
       </c>
       <c r="F224" t="n">
-        <v>2448</v>
+        <v>2445</v>
       </c>
       <c r="G224" t="n">
         <v>0</v>
@@ -6723,7 +6723,7 @@
         <v>66</v>
       </c>
       <c r="F225" t="n">
-        <v>4720</v>
+        <v>4718</v>
       </c>
       <c r="G225" t="n">
         <v>1863.56</v>
@@ -6751,7 +6751,7 @@
         <v>15</v>
       </c>
       <c r="F226" t="n">
-        <v>3547</v>
+        <v>3543</v>
       </c>
       <c r="G226" t="n">
         <v>0</v>
@@ -6807,7 +6807,7 @@
         <v>3</v>
       </c>
       <c r="F228" t="n">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="G228" t="n">
         <v>2244.92</v>
@@ -6835,7 +6835,7 @@
         <v>8</v>
       </c>
       <c r="F229" t="n">
-        <v>11963</v>
+        <v>11962</v>
       </c>
       <c r="G229" t="n">
         <v>5422.03</v>
@@ -6863,7 +6863,7 @@
         <v>52</v>
       </c>
       <c r="F230" t="n">
-        <v>5559</v>
+        <v>5557</v>
       </c>
       <c r="G230" t="n">
         <v>0</v>
@@ -6891,7 +6891,7 @@
         <v>60</v>
       </c>
       <c r="F231" t="n">
-        <v>18326</v>
+        <v>18324</v>
       </c>
       <c r="G231" t="n">
         <v>0</v>
@@ -6919,7 +6919,7 @@
         <v>97</v>
       </c>
       <c r="F232" t="n">
-        <v>24829</v>
+        <v>24821</v>
       </c>
       <c r="G232" t="n">
         <v>0</v>
@@ -6947,7 +6947,7 @@
         <v>216</v>
       </c>
       <c r="F233" t="n">
-        <v>42223</v>
+        <v>42210</v>
       </c>
       <c r="G233" t="n">
         <v>6988.97</v>
@@ -6969,13 +6969,13 @@
         </is>
       </c>
       <c r="D234" t="n">
-        <v>262.63</v>
+        <v>261.63</v>
       </c>
       <c r="E234" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F234" t="n">
-        <v>13434</v>
+        <v>13429</v>
       </c>
       <c r="G234" t="n">
         <v>1185.59</v>
@@ -7003,7 +7003,7 @@
         <v>13</v>
       </c>
       <c r="F235" t="n">
-        <v>2358</v>
+        <v>2356</v>
       </c>
       <c r="G235" t="n">
         <v>2015.26</v>
@@ -7031,7 +7031,7 @@
         <v>6</v>
       </c>
       <c r="F236" t="n">
-        <v>2315</v>
+        <v>2311</v>
       </c>
       <c r="G236" t="n">
         <v>0</v>
@@ -7059,7 +7059,7 @@
         <v>4</v>
       </c>
       <c r="F237" t="n">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G237" t="n">
         <v>3372.5</v>
@@ -7143,7 +7143,7 @@
         <v>4</v>
       </c>
       <c r="F240" t="n">
-        <v>6298</v>
+        <v>6294</v>
       </c>
       <c r="G240" t="n">
         <v>0</v>
@@ -7171,7 +7171,7 @@
         <v>10</v>
       </c>
       <c r="F241" t="n">
-        <v>3588</v>
+        <v>3581</v>
       </c>
       <c r="G241" t="n">
         <v>0</v>
@@ -7199,7 +7199,7 @@
         <v>16</v>
       </c>
       <c r="F242" t="n">
-        <v>5703</v>
+        <v>5700</v>
       </c>
       <c r="G242" t="n">
         <v>0</v>
@@ -7227,7 +7227,7 @@
         <v>16</v>
       </c>
       <c r="F243" t="n">
-        <v>5227</v>
+        <v>5225</v>
       </c>
       <c r="G243" t="n">
         <v>0</v>
@@ -7255,7 +7255,7 @@
         <v>15</v>
       </c>
       <c r="F244" t="n">
-        <v>1534</v>
+        <v>1533</v>
       </c>
       <c r="G244" t="n">
         <v>0</v>
@@ -7283,7 +7283,7 @@
         <v>60</v>
       </c>
       <c r="F245" t="n">
-        <v>7473</v>
+        <v>7470</v>
       </c>
       <c r="G245" t="n">
         <v>3388.98</v>
@@ -7311,7 +7311,7 @@
         <v>14</v>
       </c>
       <c r="F246" t="n">
-        <v>2251</v>
+        <v>2242</v>
       </c>
       <c r="G246" t="n">
         <v>0</v>
@@ -7339,7 +7339,7 @@
         <v>58</v>
       </c>
       <c r="F247" t="n">
-        <v>8621</v>
+        <v>8611</v>
       </c>
       <c r="G247" t="n">
         <v>0</v>
@@ -7395,7 +7395,7 @@
         <v>3</v>
       </c>
       <c r="F249" t="n">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="G249" t="n">
         <v>0</v>
@@ -7423,7 +7423,7 @@
         <v>4</v>
       </c>
       <c r="F250" t="n">
-        <v>1245</v>
+        <v>1242</v>
       </c>
       <c r="G250" t="n">
         <v>0</v>
@@ -7479,7 +7479,7 @@
         <v>115</v>
       </c>
       <c r="F252" t="n">
-        <v>19729</v>
+        <v>19728</v>
       </c>
       <c r="G252" t="n">
         <v>4906.8</v>
@@ -7501,13 +7501,13 @@
         </is>
       </c>
       <c r="D253" t="n">
-        <v>1235.98</v>
+        <v>1232.48</v>
       </c>
       <c r="E253" t="n">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F253" t="n">
-        <v>79846</v>
+        <v>79828</v>
       </c>
       <c r="G253" t="n">
         <v>7202.54</v>
@@ -7535,7 +7535,7 @@
         <v>0</v>
       </c>
       <c r="F254" t="n">
-        <v>558</v>
+        <v>554</v>
       </c>
       <c r="G254" t="n">
         <v>0</v>
@@ -7563,7 +7563,7 @@
         <v>143</v>
       </c>
       <c r="F255" t="n">
-        <v>16013</v>
+        <v>16010</v>
       </c>
       <c r="G255" t="n">
         <v>3108.47</v>
@@ -7591,7 +7591,7 @@
         <v>130</v>
       </c>
       <c r="F256" t="n">
-        <v>36786</v>
+        <v>36784</v>
       </c>
       <c r="G256" t="n">
         <v>0</v>
@@ -7619,7 +7619,7 @@
         <v>10</v>
       </c>
       <c r="F257" t="n">
-        <v>4096</v>
+        <v>4090</v>
       </c>
       <c r="G257" t="n">
         <v>0</v>
@@ -7641,13 +7641,13 @@
         </is>
       </c>
       <c r="D258" t="n">
-        <v>144.84</v>
+        <v>142.13</v>
       </c>
       <c r="E258" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F258" t="n">
-        <v>10252</v>
+        <v>10240</v>
       </c>
       <c r="G258" t="n">
         <v>769.49</v>
@@ -7669,13 +7669,13 @@
         </is>
       </c>
       <c r="D259" t="n">
-        <v>538.9400000000001</v>
+        <v>535.77</v>
       </c>
       <c r="E259" t="n">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F259" t="n">
-        <v>15503</v>
+        <v>15495</v>
       </c>
       <c r="G259" t="n">
         <v>0</v>
@@ -7703,7 +7703,7 @@
         <v>9</v>
       </c>
       <c r="F260" t="n">
-        <v>1464</v>
+        <v>1462</v>
       </c>
       <c r="G260" t="n">
         <v>0</v>
@@ -7725,13 +7725,13 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>126.1</v>
+        <v>125.1</v>
       </c>
       <c r="E261" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F261" t="n">
-        <v>10352</v>
+        <v>10348</v>
       </c>
       <c r="G261" t="n">
         <v>0</v>
@@ -7759,7 +7759,7 @@
         <v>38</v>
       </c>
       <c r="F262" t="n">
-        <v>3261</v>
+        <v>3260</v>
       </c>
       <c r="G262" t="n">
         <v>0</v>
@@ -7787,7 +7787,7 @@
         <v>16</v>
       </c>
       <c r="F263" t="n">
-        <v>4989</v>
+        <v>4983</v>
       </c>
       <c r="G263" t="n">
         <v>0</v>
@@ -7815,7 +7815,7 @@
         <v>22</v>
       </c>
       <c r="F264" t="n">
-        <v>1978</v>
+        <v>1977</v>
       </c>
       <c r="G264" t="n">
         <v>0</v>
@@ -7843,7 +7843,7 @@
         <v>25</v>
       </c>
       <c r="F265" t="n">
-        <v>4419</v>
+        <v>4418</v>
       </c>
       <c r="G265" t="n">
         <v>5196.61</v>
@@ -7899,7 +7899,7 @@
         <v>114</v>
       </c>
       <c r="F267" t="n">
-        <v>14634</v>
+        <v>14627</v>
       </c>
       <c r="G267" t="n">
         <v>3219.49</v>
@@ -7927,7 +7927,7 @@
         <v>3</v>
       </c>
       <c r="F268" t="n">
-        <v>597</v>
+        <v>594</v>
       </c>
       <c r="G268" t="n">
         <v>0</v>
@@ -7949,13 +7949,13 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>373.24</v>
+        <v>369.74</v>
       </c>
       <c r="E269" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F269" t="n">
-        <v>17952</v>
+        <v>17942</v>
       </c>
       <c r="G269" t="n">
         <v>8473.73</v>
@@ -7983,7 +7983,7 @@
         <v>18</v>
       </c>
       <c r="F270" t="n">
-        <v>3685</v>
+        <v>3680</v>
       </c>
       <c r="G270" t="n">
         <v>0</v>
@@ -8039,7 +8039,7 @@
         <v>6</v>
       </c>
       <c r="F272" t="n">
-        <v>1496</v>
+        <v>1495</v>
       </c>
       <c r="G272" t="n">
         <v>0</v>
@@ -8067,7 +8067,7 @@
         <v>2</v>
       </c>
       <c r="F273" t="n">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="G273" t="n">
         <v>0</v>
@@ -8095,7 +8095,7 @@
         <v>50</v>
       </c>
       <c r="F274" t="n">
-        <v>6957</v>
+        <v>6955</v>
       </c>
       <c r="G274" t="n">
         <v>0</v>
@@ -8151,7 +8151,7 @@
         <v>34</v>
       </c>
       <c r="F276" t="n">
-        <v>8246</v>
+        <v>8240</v>
       </c>
       <c r="G276" t="n">
         <v>0</v>
@@ -8179,7 +8179,7 @@
         <v>4</v>
       </c>
       <c r="F277" t="n">
-        <v>3370</v>
+        <v>3369</v>
       </c>
       <c r="G277" t="n">
         <v>380.51</v>
@@ -8207,7 +8207,7 @@
         <v>125</v>
       </c>
       <c r="F278" t="n">
-        <v>11716</v>
+        <v>11705</v>
       </c>
       <c r="G278" t="n">
         <v>4066.95</v>
@@ -8235,7 +8235,7 @@
         <v>59</v>
       </c>
       <c r="F279" t="n">
-        <v>6094</v>
+        <v>6091</v>
       </c>
       <c r="G279" t="n">
         <v>0</v>
@@ -8263,7 +8263,7 @@
         <v>54</v>
       </c>
       <c r="F280" t="n">
-        <v>10254</v>
+        <v>10249</v>
       </c>
       <c r="G280" t="n">
         <v>0</v>
@@ -8291,7 +8291,7 @@
         <v>4</v>
       </c>
       <c r="F281" t="n">
-        <v>5501</v>
+        <v>5498</v>
       </c>
       <c r="G281" t="n">
         <v>0</v>
@@ -8319,7 +8319,7 @@
         <v>8</v>
       </c>
       <c r="F282" t="n">
-        <v>3384</v>
+        <v>3381</v>
       </c>
       <c r="G282" t="n">
         <v>0</v>
@@ -8347,7 +8347,7 @@
         <v>38</v>
       </c>
       <c r="F283" t="n">
-        <v>4572</v>
+        <v>4567</v>
       </c>
       <c r="G283" t="n">
         <v>0</v>
@@ -8431,7 +8431,7 @@
         <v>4</v>
       </c>
       <c r="F286" t="n">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="G286" t="n">
         <v>0</v>
@@ -8481,13 +8481,13 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>3319.99</v>
+        <v>3314.04</v>
       </c>
       <c r="E288" t="n">
-        <v>1203</v>
+        <v>1199</v>
       </c>
       <c r="F288" t="n">
-        <v>109621</v>
+        <v>109589</v>
       </c>
       <c r="G288" t="n">
         <v>21199.99</v>
@@ -8537,13 +8537,13 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>978.34</v>
+        <v>971.79</v>
       </c>
       <c r="E290" t="n">
-        <v>450</v>
+        <v>444</v>
       </c>
       <c r="F290" t="n">
-        <v>42729</v>
+        <v>42713</v>
       </c>
       <c r="G290" t="n">
         <v>0</v>
@@ -8565,13 +8565,13 @@
         </is>
       </c>
       <c r="D291" t="n">
-        <v>978.16</v>
+        <v>974.74</v>
       </c>
       <c r="E291" t="n">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="F291" t="n">
-        <v>32401</v>
+        <v>32382</v>
       </c>
       <c r="G291" t="n">
         <v>28216.11</v>
@@ -8599,7 +8599,7 @@
         <v>634</v>
       </c>
       <c r="F292" t="n">
-        <v>57023</v>
+        <v>57008</v>
       </c>
       <c r="G292" t="n">
         <v>7033.05</v>
@@ -8655,7 +8655,7 @@
         <v>198</v>
       </c>
       <c r="F294" t="n">
-        <v>28621</v>
+        <v>28609</v>
       </c>
       <c r="G294" t="n">
         <v>0</v>
@@ -8683,7 +8683,7 @@
         <v>87</v>
       </c>
       <c r="F295" t="n">
-        <v>8688</v>
+        <v>8687</v>
       </c>
       <c r="G295" t="n">
         <v>4236.44</v>
@@ -8711,7 +8711,7 @@
         <v>35</v>
       </c>
       <c r="F296" t="n">
-        <v>5276</v>
+        <v>5274</v>
       </c>
       <c r="G296" t="n">
         <v>0</v>
@@ -8733,13 +8733,13 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>562.14</v>
+        <v>561.14</v>
       </c>
       <c r="E297" t="n">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F297" t="n">
-        <v>18148</v>
+        <v>18143</v>
       </c>
       <c r="G297" t="n">
         <v>4660.17</v>
@@ -8767,7 +8767,7 @@
         <v>106</v>
       </c>
       <c r="F298" t="n">
-        <v>15879</v>
+        <v>15876</v>
       </c>
       <c r="G298" t="n">
         <v>0</v>
@@ -8795,7 +8795,7 @@
         <v>545</v>
       </c>
       <c r="F299" t="n">
-        <v>46652</v>
+        <v>46647</v>
       </c>
       <c r="G299" t="n">
         <v>5931.36</v>
@@ -8823,7 +8823,7 @@
         <v>444</v>
       </c>
       <c r="F300" t="n">
-        <v>67175</v>
+        <v>67174</v>
       </c>
       <c r="G300" t="n">
         <v>24572.88</v>
@@ -8851,7 +8851,7 @@
         <v>765</v>
       </c>
       <c r="F301" t="n">
-        <v>80065</v>
+        <v>80064</v>
       </c>
       <c r="G301" t="n">
         <v>5931.36</v>
@@ -8901,13 +8901,13 @@
         </is>
       </c>
       <c r="D303" t="n">
-        <v>268.97</v>
+        <v>261.72</v>
       </c>
       <c r="E303" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F303" t="n">
-        <v>3528</v>
+        <v>3527</v>
       </c>
       <c r="G303" t="n">
         <v>9829.66</v>
@@ -8991,7 +8991,7 @@
         <v>83</v>
       </c>
       <c r="F306" t="n">
-        <v>19242</v>
+        <v>19240</v>
       </c>
       <c r="G306" t="n">
         <v>7626.27</v>
@@ -9019,7 +9019,7 @@
         <v>142</v>
       </c>
       <c r="F307" t="n">
-        <v>17424</v>
+        <v>17422</v>
       </c>
       <c r="G307" t="n">
         <v>5931.36</v>
@@ -9131,7 +9131,7 @@
         <v>210</v>
       </c>
       <c r="F311" t="n">
-        <v>7436</v>
+        <v>7434</v>
       </c>
       <c r="G311" t="n">
         <v>18976.25</v>
@@ -9159,7 +9159,7 @@
         <v>193</v>
       </c>
       <c r="F312" t="n">
-        <v>11576</v>
+        <v>11573</v>
       </c>
       <c r="G312" t="n">
         <v>0</v>
@@ -9187,7 +9187,7 @@
         <v>276</v>
       </c>
       <c r="F313" t="n">
-        <v>18933</v>
+        <v>18931</v>
       </c>
       <c r="G313" t="n">
         <v>12540.68</v>
@@ -9215,7 +9215,7 @@
         <v>160</v>
       </c>
       <c r="F314" t="n">
-        <v>17523</v>
+        <v>17521</v>
       </c>
       <c r="G314" t="n">
         <v>2372.03</v>
@@ -9243,7 +9243,7 @@
         <v>141</v>
       </c>
       <c r="F315" t="n">
-        <v>7147</v>
+        <v>7146</v>
       </c>
       <c r="G315" t="n">
         <v>4744.06</v>
@@ -9271,7 +9271,7 @@
         <v>243</v>
       </c>
       <c r="F316" t="n">
-        <v>15353</v>
+        <v>15350</v>
       </c>
       <c r="G316" t="n">
         <v>11735.6</v>
@@ -9321,13 +9321,13 @@
         </is>
       </c>
       <c r="D318" t="n">
-        <v>764.73</v>
+        <v>762.14</v>
       </c>
       <c r="E318" t="n">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F318" t="n">
-        <v>18121</v>
+        <v>18114</v>
       </c>
       <c r="G318" t="n">
         <v>9405.08</v>
@@ -9775,7 +9775,7 @@
         <v>152</v>
       </c>
       <c r="F334" t="n">
-        <v>23089</v>
+        <v>23082</v>
       </c>
       <c r="G334" t="n">
         <v>0</v>
@@ -9803,7 +9803,7 @@
         <v>16</v>
       </c>
       <c r="F335" t="n">
-        <v>7548</v>
+        <v>7542</v>
       </c>
       <c r="G335" t="n">
         <v>0</v>
@@ -9831,7 +9831,7 @@
         <v>483</v>
       </c>
       <c r="F336" t="n">
-        <v>43170</v>
+        <v>43166</v>
       </c>
       <c r="G336" t="n">
         <v>49128.04</v>
@@ -9887,7 +9887,7 @@
         <v>29</v>
       </c>
       <c r="F338" t="n">
-        <v>9752</v>
+        <v>9751</v>
       </c>
       <c r="G338" t="n">
         <v>0</v>
@@ -10307,7 +10307,7 @@
         <v>28</v>
       </c>
       <c r="F353" t="n">
-        <v>2352</v>
+        <v>2351</v>
       </c>
       <c r="G353" t="n">
         <v>8259.18</v>
@@ -10699,7 +10699,7 @@
         <v>60</v>
       </c>
       <c r="F367" t="n">
-        <v>13634</v>
+        <v>13631</v>
       </c>
       <c r="G367" t="n">
         <v>1100.85</v>
@@ -11035,7 +11035,7 @@
         <v>20</v>
       </c>
       <c r="F379" t="n">
-        <v>6006</v>
+        <v>6005</v>
       </c>
       <c r="G379" t="n">
         <v>6946.6</v>
@@ -11427,7 +11427,7 @@
         <v>312</v>
       </c>
       <c r="F393" t="n">
-        <v>48608</v>
+        <v>48604</v>
       </c>
       <c r="G393" t="n">
         <v>15714.44</v>
@@ -11483,7 +11483,7 @@
         <v>46</v>
       </c>
       <c r="F395" t="n">
-        <v>10014</v>
+        <v>10011</v>
       </c>
       <c r="G395" t="n">
         <v>2897.46</v>
@@ -11539,7 +11539,7 @@
         <v>141</v>
       </c>
       <c r="F397" t="n">
-        <v>20533</v>
+        <v>20531</v>
       </c>
       <c r="G397" t="n">
         <v>2032.2</v>
@@ -11567,7 +11567,7 @@
         <v>367</v>
       </c>
       <c r="F398" t="n">
-        <v>48370</v>
+        <v>48369</v>
       </c>
       <c r="G398" t="n">
         <v>7163.55</v>
@@ -15823,7 +15823,7 @@
         <v>79</v>
       </c>
       <c r="F550" t="n">
-        <v>5020</v>
+        <v>5019</v>
       </c>
       <c r="G550" t="n">
         <v>0</v>
@@ -15879,7 +15879,7 @@
         <v>223</v>
       </c>
       <c r="F552" t="n">
-        <v>16838</v>
+        <v>16837</v>
       </c>
       <c r="G552" t="n">
         <v>0</v>
@@ -16971,7 +16971,7 @@
         <v>366</v>
       </c>
       <c r="F5" t="n">
-        <v>102311</v>
+        <v>102291</v>
       </c>
       <c r="G5" t="n">
         <v>16267.8</v>
@@ -16999,7 +16999,7 @@
         <v>185</v>
       </c>
       <c r="F6" t="n">
-        <v>42948</v>
+        <v>42946</v>
       </c>
       <c r="G6" t="n">
         <v>8470.35</v>
@@ -17195,7 +17195,7 @@
         <v>366</v>
       </c>
       <c r="F13" t="n">
-        <v>87199</v>
+        <v>87129</v>
       </c>
       <c r="G13" t="n">
         <v>24401.69</v>
@@ -17581,13 +17581,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1634.84</v>
+        <v>1633.82</v>
       </c>
       <c r="E27" t="n">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="F27" t="n">
-        <v>170262</v>
+        <v>170258</v>
       </c>
       <c r="G27" t="n">
         <v>1355.08</v>
@@ -17811,7 +17811,7 @@
         <v>68</v>
       </c>
       <c r="F35" t="n">
-        <v>12448</v>
+        <v>12447</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
@@ -17917,13 +17917,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>6877.2</v>
+        <v>6870.05</v>
       </c>
       <c r="E39" t="n">
-        <v>3012</v>
+        <v>3007</v>
       </c>
       <c r="F39" t="n">
-        <v>794866</v>
+        <v>794865</v>
       </c>
       <c r="G39" t="n">
         <v>29992.38</v>

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-06-14
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,42 +419,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -17231,42 +17219,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -18519,47 +18507,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-08-10
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SP" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SD" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="SD" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SB" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,42 +419,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -17231,42 +17219,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -18519,47 +18507,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>

</xml_diff>

<commit_message>
chore(weekly-sync): auto-pull through 2026-08-31
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
+++ b/data/ams_weekly_data/Audio_Array/ads_report_week21.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -36,7 +39,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -44,12 +47,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,42 +431,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -17219,42 +17231,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
@@ -18507,47 +18519,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Portfolio name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Campaign Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Advertised ASIN</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Impressions</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Clicks</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>14 Day Total Sales (₹)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>14 Day Total Units (#)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>

</xml_diff>